<commit_message>
feat(spec-parser): add full artwork spec sheet parser, annotation font matcher, and ROI auto-crop
</commit_message>
<xml_diff>
--- a/sample_data/1000341139_Loveskin-PT_001.xlsx
+++ b/sample_data/1000341139_Loveskin-PT_001.xlsx
@@ -435,8 +435,8 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -544,17 +544,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1000341139-PT</t>
+          <t>Z5E213TS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Midnight Navy</t>
+          <t>Nero</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -611,17 +611,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1000341139-PT</t>
+          <t>Z5E213TS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Midnight Navy</t>
+          <t>Nero</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -678,17 +678,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1000341139-PT</t>
+          <t>Z5E213TS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Midnight Navy</t>
+          <t>Nero</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H4" t="n">

</xml_diff>